<commit_message>
Updated excel sheet with new records
</commit_message>
<xml_diff>
--- a/boundaries.xlsx
+++ b/boundaries.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="89">
   <si>
     <t>book_name</t>
   </si>
@@ -148,6 +148,144 @@
   </si>
   <si>
     <t>aptavani-4_hindi.pdf</t>
+  </si>
+  <si>
+    <t>aptavani-5_hindi.pdf</t>
+  </si>
+  <si>
+    <t>aptavani-6_hindi.pdf</t>
+  </si>
+  <si>
+    <t>aptavani-7_hindi.pdf</t>
+  </si>
+  <si>
+    <t>aptavani-8_hindi.pdf</t>
+  </si>
+  <si>
+    <t>aptavani-9_hindi.pdf</t>
+  </si>
+  <si>
+    <t>Chamatkar_hindi.pdf</t>
+  </si>
+  <si>
+    <t>dada_kaun_hindi.pdf</t>
+  </si>
+  <si>
+    <t>gnani-purush.pdf</t>
+  </si>
+  <si>
+    <t>guru_shishya.pdf</t>
+  </si>
+  <si>
+    <t>Gyani-Purursh-Bhag-1_hindi.pdf</t>
+  </si>
+  <si>
+    <t>karma.pdf</t>
+  </si>
+  <si>
+    <t>paap-punya_hindi.pdf</t>
+  </si>
+  <si>
+    <t>pahchane-antharan-ko-hindi.pdf</t>
+  </si>
+  <si>
+    <t>Paiso-Ka-Vyavhar(granth).pdf</t>
+  </si>
+  <si>
+    <t>Pratikraman-granth_hindi.pdf</t>
+  </si>
+  <si>
+    <t>Sahajta_hindi.pdf</t>
+  </si>
+  <si>
+    <t>Satya-Asatya-Hindi.pdf</t>
+  </si>
+  <si>
+    <t>Seva-paropkar.pdf</t>
+  </si>
+  <si>
+    <t>Shri-Simandhar-Swami-meduim.pdf</t>
+  </si>
+  <si>
+    <t>simandhar-swami.pdf</t>
+  </si>
+  <si>
+    <t>trimantra_hindi.pdf</t>
+  </si>
+  <si>
+    <t>Vaani-Vyvahaar-Me_hindi.pdf</t>
+  </si>
+  <si>
+    <t>Aatm-Sakshatkar.pdf</t>
+  </si>
+  <si>
+    <t>gujarati</t>
+  </si>
+  <si>
+    <t>Adjust-Everywhere.pdf</t>
+  </si>
+  <si>
+    <t>Banyu-te-j-nyay.pdf</t>
+  </si>
+  <si>
+    <t>Athadamal-Talo.pdf</t>
+  </si>
+  <si>
+    <t>Bhogve-eni-bhul.pdf</t>
+  </si>
+  <si>
+    <t>Chinta.pdf</t>
+  </si>
+  <si>
+    <t>Hu-kon-chhu.pdf</t>
+  </si>
+  <si>
+    <t>Klesh-Vinanu-Jivan.pdf</t>
+  </si>
+  <si>
+    <t>Maa-bap-chhokarano-vyavahar.pdf</t>
+  </si>
+  <si>
+    <t>Prem.pdf</t>
+  </si>
+  <si>
+    <t>krodh.pdf</t>
+  </si>
+  <si>
+    <t>Pratikraman.pdf</t>
+  </si>
+  <si>
+    <t>Chamatkar.pdf</t>
+  </si>
+  <si>
+    <t>Daan.pdf</t>
+  </si>
+  <si>
+    <t>Dadabhagwan-kon.pdf</t>
+  </si>
+  <si>
+    <t>Gurushishya.pdf</t>
+  </si>
+  <si>
+    <t>Karm-nu-vignan.pdf</t>
+  </si>
+  <si>
+    <t>Manav-dharma.pdf</t>
+  </si>
+  <si>
+    <t>Mrutyu-tana-rahasyo.pdf</t>
+  </si>
+  <si>
+    <t>Nijdosh-darsahn-thi-nirdosh.pdf</t>
+  </si>
+  <si>
+    <t>Paisa-no-vyavahar-sankshipt.pdf</t>
+  </si>
+  <si>
+    <t>Pati-patni-no-divya-vyavahar.pdf</t>
+  </si>
+  <si>
+    <t>Trimantra.pdf</t>
   </si>
 </sst>
 </file>
@@ -487,11 +625,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1040,6 +1177,636 @@
         <v>377</v>
       </c>
     </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40">
+        <v>32</v>
+      </c>
+      <c r="D40">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>44</v>
+      </c>
+      <c r="B41" t="s">
+        <v>5</v>
+      </c>
+      <c r="C41">
+        <v>26</v>
+      </c>
+      <c r="D41">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>45</v>
+      </c>
+      <c r="B42" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42">
+        <v>42</v>
+      </c>
+      <c r="D42">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>46</v>
+      </c>
+      <c r="B43" t="s">
+        <v>5</v>
+      </c>
+      <c r="C43">
+        <v>40</v>
+      </c>
+      <c r="D43">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>47</v>
+      </c>
+      <c r="B44" t="s">
+        <v>5</v>
+      </c>
+      <c r="C44">
+        <v>52</v>
+      </c>
+      <c r="D44">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>48</v>
+      </c>
+      <c r="B45" t="s">
+        <v>5</v>
+      </c>
+      <c r="C45">
+        <v>10</v>
+      </c>
+      <c r="D45">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>49</v>
+      </c>
+      <c r="B46" t="s">
+        <v>5</v>
+      </c>
+      <c r="C46">
+        <v>10</v>
+      </c>
+      <c r="D46">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>50</v>
+      </c>
+      <c r="B47" t="s">
+        <v>5</v>
+      </c>
+      <c r="C47">
+        <v>36</v>
+      </c>
+      <c r="D47">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>51</v>
+      </c>
+      <c r="B48" t="s">
+        <v>5</v>
+      </c>
+      <c r="C48">
+        <v>12</v>
+      </c>
+      <c r="D48">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B49" t="s">
+        <v>5</v>
+      </c>
+      <c r="C49">
+        <v>66</v>
+      </c>
+      <c r="D49">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>53</v>
+      </c>
+      <c r="B50" t="s">
+        <v>5</v>
+      </c>
+      <c r="C50">
+        <v>10</v>
+      </c>
+      <c r="D50">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>54</v>
+      </c>
+      <c r="B51" t="s">
+        <v>5</v>
+      </c>
+      <c r="C51">
+        <v>10</v>
+      </c>
+      <c r="D51">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>55</v>
+      </c>
+      <c r="B52" t="s">
+        <v>5</v>
+      </c>
+      <c r="C52">
+        <v>10</v>
+      </c>
+      <c r="D52">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53" t="s">
+        <v>5</v>
+      </c>
+      <c r="C53">
+        <v>74</v>
+      </c>
+      <c r="D53">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>57</v>
+      </c>
+      <c r="B54" t="s">
+        <v>5</v>
+      </c>
+      <c r="C54">
+        <v>56</v>
+      </c>
+      <c r="D54">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>58</v>
+      </c>
+      <c r="B55" t="s">
+        <v>5</v>
+      </c>
+      <c r="C55">
+        <v>38</v>
+      </c>
+      <c r="D55">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" t="s">
+        <v>5</v>
+      </c>
+      <c r="C56">
+        <v>10</v>
+      </c>
+      <c r="D56">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>60</v>
+      </c>
+      <c r="B57" t="s">
+        <v>5</v>
+      </c>
+      <c r="C57">
+        <v>8</v>
+      </c>
+      <c r="D57">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>61</v>
+      </c>
+      <c r="B58" t="s">
+        <v>5</v>
+      </c>
+      <c r="C58">
+        <v>22</v>
+      </c>
+      <c r="D58">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>62</v>
+      </c>
+      <c r="B59" t="s">
+        <v>5</v>
+      </c>
+      <c r="C59">
+        <v>12</v>
+      </c>
+      <c r="D59">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>63</v>
+      </c>
+      <c r="B60" t="s">
+        <v>5</v>
+      </c>
+      <c r="C60">
+        <v>10</v>
+      </c>
+      <c r="D60">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>64</v>
+      </c>
+      <c r="B61" t="s">
+        <v>5</v>
+      </c>
+      <c r="C61">
+        <v>12</v>
+      </c>
+      <c r="D61">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>65</v>
+      </c>
+      <c r="B62" t="s">
+        <v>66</v>
+      </c>
+      <c r="C62">
+        <v>4</v>
+      </c>
+      <c r="D62">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>67</v>
+      </c>
+      <c r="B63" t="s">
+        <v>66</v>
+      </c>
+      <c r="C63">
+        <v>8</v>
+      </c>
+      <c r="D63">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>68</v>
+      </c>
+      <c r="B64" t="s">
+        <v>66</v>
+      </c>
+      <c r="C64">
+        <v>8</v>
+      </c>
+      <c r="D64">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>69</v>
+      </c>
+      <c r="B65" t="s">
+        <v>66</v>
+      </c>
+      <c r="C65">
+        <v>8</v>
+      </c>
+      <c r="D65">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>70</v>
+      </c>
+      <c r="B66" t="s">
+        <v>66</v>
+      </c>
+      <c r="C66">
+        <v>8</v>
+      </c>
+      <c r="D66">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>71</v>
+      </c>
+      <c r="B67" t="s">
+        <v>66</v>
+      </c>
+      <c r="C67">
+        <v>8</v>
+      </c>
+      <c r="D67">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>72</v>
+      </c>
+      <c r="B68" t="s">
+        <v>66</v>
+      </c>
+      <c r="C68">
+        <v>8</v>
+      </c>
+      <c r="D68">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>73</v>
+      </c>
+      <c r="B69" t="s">
+        <v>66</v>
+      </c>
+      <c r="C69">
+        <v>10</v>
+      </c>
+      <c r="D69">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>74</v>
+      </c>
+      <c r="B70" t="s">
+        <v>66</v>
+      </c>
+      <c r="C70">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>75</v>
+      </c>
+      <c r="B71" t="s">
+        <v>66</v>
+      </c>
+      <c r="C71">
+        <v>8</v>
+      </c>
+      <c r="D71">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>76</v>
+      </c>
+      <c r="B72" t="s">
+        <v>66</v>
+      </c>
+      <c r="C72">
+        <v>8</v>
+      </c>
+      <c r="D72">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>77</v>
+      </c>
+      <c r="B73" t="s">
+        <v>66</v>
+      </c>
+      <c r="C73">
+        <v>12</v>
+      </c>
+      <c r="D73">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>78</v>
+      </c>
+      <c r="B74" t="s">
+        <v>66</v>
+      </c>
+      <c r="C74">
+        <v>8</v>
+      </c>
+      <c r="D74">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>79</v>
+      </c>
+      <c r="B75" t="s">
+        <v>66</v>
+      </c>
+      <c r="C75">
+        <v>8</v>
+      </c>
+      <c r="D75">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>80</v>
+      </c>
+      <c r="B76" t="s">
+        <v>66</v>
+      </c>
+      <c r="C76">
+        <v>10</v>
+      </c>
+      <c r="D76">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>81</v>
+      </c>
+      <c r="B77" t="s">
+        <v>66</v>
+      </c>
+      <c r="C77">
+        <v>8</v>
+      </c>
+      <c r="D77">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>82</v>
+      </c>
+      <c r="B78" t="s">
+        <v>66</v>
+      </c>
+      <c r="C78">
+        <v>10</v>
+      </c>
+      <c r="D78">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>83</v>
+      </c>
+      <c r="B79" t="s">
+        <v>66</v>
+      </c>
+      <c r="C79">
+        <v>10</v>
+      </c>
+      <c r="D79">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>84</v>
+      </c>
+      <c r="B80" t="s">
+        <v>66</v>
+      </c>
+      <c r="C80">
+        <v>10</v>
+      </c>
+      <c r="D80">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>85</v>
+      </c>
+      <c r="B81" t="s">
+        <v>66</v>
+      </c>
+      <c r="C81">
+        <v>20</v>
+      </c>
+      <c r="D81">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>86</v>
+      </c>
+      <c r="B82" t="s">
+        <v>66</v>
+      </c>
+      <c r="C82">
+        <v>10</v>
+      </c>
+      <c r="D82">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>87</v>
+      </c>
+      <c r="B83" t="s">
+        <v>66</v>
+      </c>
+      <c r="C83">
+        <v>12</v>
+      </c>
+      <c r="D83">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>88</v>
+      </c>
+      <c r="B84" t="s">
+        <v>66</v>
+      </c>
+      <c r="C84">
+        <v>8</v>
+      </c>
+      <c r="D84">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>